<commit_message>
Consolidate w2-ai-product into root marimo workflow
</commit_message>
<xml_diff>
--- a/w2-ai-product/outputs/assignment_01.xlsx
+++ b/w2-ai-product/outputs/assignment_01.xlsx
@@ -523,7 +523,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>features: A17 Pro chip, 120 Hz ProMotion display, USB‑C fast charging; dimensions: compact</t>
+          <t>features: A17 Pro chip, 120 Hz ProMotion display, USB‑C fast charging; dimensions: compact</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -538,24 +538,24 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Experience the future of smartphone technology with the Apple iPhone 15 Pro. Powered by the lightning-fast A17 Pro chip, this device delivers seamless performance and efficient battery life. Enjoy a stunning 120Hz ProMotion display that brings your content to life. With a compact design and durable titanium frame, the iPhone 15 Pro is built to last. Plus, fast charging via USB-C gets you back to 100% in no time. Protected by Ceramic Shield glass and a 1-year limited warranty, this phone is a reliable companion for your daily adventures.</t>
+          <t>Experience the future of smartphones with the Apple iPhone 15 Pro. Powered by the lightning-fast A17 Pro chip, this device delivers seamless performance and effortless multitasking. The stunning 120 Hz ProMotion display brings vibrant colors and silky-smooth visuals to life. With a compact design and durable titanium frame, plus Ceramic Shield glass for added protection, this iPhone is both stylish and resilient. Enjoy fast charging via USB-C and peace of mind with a 1-year limited warranty.</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>8572</v>
+        <v>5156.2</v>
       </c>
       <c r="G2" t="n">
         <v>214</v>
       </c>
       <c r="H2" t="n">
-        <v>112</v>
+        <v>97</v>
       </c>
       <c r="I2" t="n">
-        <v>1.1e-05</v>
+        <v>1.01e-05</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>good</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -602,7 +602,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>features: 200 MP camera, S‑Pen support, 120 Hz AMOLED; sustainably sourced</t>
+          <t>features: 200 MP camera, S‑Pen support, 120 Hz AMOLED; sustainably sourced</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -617,20 +617,20 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Elevate your mobile experience with the Samsung Galaxy S24 Ultra. Capture life's moments in stunning detail with its 200MP camera, while the S-Pen lets you express your creativity. Enjoy seamless visuals on the 120Hz AMOLED display. Built with a durable Armor Aluminum frame and Gorilla Glass Victus, this phone is designed to withstand the demands of everyday use. Plus, its sustainably sourced materials give you peace of mind. Backed by a 1-year limited warranty, you can trust the S24 Ultra to deliver.</t>
+          <t>Capture life's moments with unparalleled clarity and precision. The Samsung Galaxy S24 Ultra boasts a 200MP camera, perfect for capturing the world's beauty in stunning detail. The S-Pen support lets you express yourself freely, while the 120Hz AMOLED display brings your content to life. Built with sustainably sourced materials and a durable Armor Aluminum frame, this phone is both eco-friendly and long-lasting. Enjoy peace of mind with our 1-year limited warranty.</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>5682.3</v>
+        <v>1899.5</v>
       </c>
       <c r="G3" t="n">
         <v>217</v>
       </c>
       <c r="H3" t="n">
-        <v>112</v>
+        <v>96</v>
       </c>
       <c r="I3" t="n">
-        <v>1.11e-05</v>
+        <v>1.01e-05</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
@@ -654,12 +654,12 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>bad</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>bad</t>
+          <t>good</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
@@ -681,7 +681,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>features: Tensor G3 chip, Magic Eraser, 50 MP camera; rating: 4.7/5</t>
+          <t>features: Tensor G3 chip, Magic Eraser, 50 MP camera; rating: 4.7/5</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -696,20 +696,20 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Capture life's moments with the Google Pixel 8 Pro, featuring the powerful Tensor G3 chip for seamless performance. Its advanced 50MP camera, paired with Magic Eraser, lets you edit out unwanted objects with ease. The device's durable design boasts a matte glass back and aluminum frame, built to withstand daily wear. With a 4.7/5 rating, you can trust the Pixel 8 Pro to deliver exceptional results. Enjoy peace of mind with a 1-year limited warranty.</t>
+          <t>Capture life's moments with the Google Pixel 8 Pro, featuring the powerful Tensor G3 chip for seamless performance. Its advanced 50MP camera, paired with Magic Eraser, lets you edit out unwanted objects and backgrounds with ease. The sleek design boasts a matte glass back and sturdy aluminum frame. With a 4.7/5 rating, this phone has earned the trust of many. Plus, enjoy peace of mind with a 1-year limited warranty.</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>4949.9</v>
+        <v>2399.7</v>
       </c>
       <c r="G4" t="n">
         <v>215</v>
       </c>
       <c r="H4" t="n">
-        <v>101</v>
+        <v>94</v>
       </c>
       <c r="I4" t="n">
-        <v>1.04e-05</v>
+        <v>9.94e-06</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
@@ -760,7 +760,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>features: active noise cancelling, 30 hr battery, Bluetooth 5.2; capacity: large</t>
+          <t>features: active noise cancelling, 30 hr battery, Bluetooth 5.2; capacity: large</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -775,24 +775,24 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Immerse yourself in pure sound with the Sony WH-1000XM5 Headphones. These premium headphones boast advanced active noise cancelling technology, ensuring you can focus on your music without distractions. Enjoy up to 30 hours of uninterrupted listening on a single charge, thanks to their long-lasting battery. With Bluetooth 5.2 connectivity, you can seamlessly pair with your devices. The large synthetic leather earcups provide comfort during extended wear. Backed by a 1-year limited warranty, you can trust these headphones to deliver exceptional sound and value.</t>
+          <t>Immerse yourself in pure sound with the Sony WH-1000XM5 Headphones. These premium headphones boast active noise cancelling technology, ensuring you're fully engaged in your music, podcasts, or calls. Enjoy up to 30 hours of uninterrupted listening on a single charge, and seamlessly connect via Bluetooth 5.2. The large capacity and synthetic leather earcups provide all-day comfort. With a 1-year limited warranty, you can trust your investment in exceptional sound.</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>4303.5</v>
+        <v>4320.1</v>
       </c>
       <c r="G5" t="n">
         <v>214</v>
       </c>
       <c r="H5" t="n">
-        <v>112</v>
+        <v>98</v>
       </c>
       <c r="I5" t="n">
-        <v>1.1e-05</v>
+        <v>1.016e-05</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>good</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -854,20 +854,20 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Immerse yourself in pure sound with the Bose QuietComfort Ultra Earbuds. These award-winning earbuds feature CustomTune sound calibration, ensuring a tailored listening experience that adapts to your unique hearing. Advanced Noise Cancellation (ANC) blocks out distractions, while the IPX4 rating keeps them protected from sweat and water. With silicone ear tips for a comfortable fit, you can enjoy your favorite music, podcasts, or audiobooks in crystal-clear quality.</t>
+          <t>Immerse yourself in pure sound with the Bose QuietComfort Ultra Earbuds. These award-winning earbuds feature CustomTune sound calibration, expertly tuning the sound to your unique hearing. Active Noise Cancellation (ANC) blocks out distractions, while IPX4-rated silicone ear tips keep you listening in comfort. With a 1-year limited warranty, you can enjoy your music with confidence. Experience the perfect blend of sound and style with the QuietComfort Ultra Earbuds.</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>2726.2</v>
+        <v>4414.3</v>
       </c>
       <c r="G6" t="n">
         <v>208</v>
       </c>
       <c r="H6" t="n">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="I6" t="n">
-        <v>9.92e-06</v>
+        <v>1.01e-05</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
@@ -933,20 +933,20 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Meet the Amazon Echo Dot (5th Gen), your smart home's new best friend. With Alexa by your side, control lights, play music, and get answers to your burning questions. This compact powerhouse also monitors the temperature, ensuring your space is always just right. Plus, enjoy richer sound with improved bass. And, with its eco-friendly recycled fabric mesh, you can feel good about your purchase. Backed by a 1-year limited warranty, the Echo Dot is the perfect blend of style, substance, and sustainability.</t>
+          <t>Meet the Amazon Echo Dot (5th Gen), a compact smart speaker that's not only stylish but also sustainable. Made from recycled fabric mesh, you can feel good about your purchase. With Alexa built-in, you can control your home, play music, and get answers to your questions with just your voice. Plus, enjoy improved bass and a temperature sensor for added convenience. Backed by a 1-year limited warranty, you can trust that your Echo Dot will keep on performing.</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>2955.7</v>
+        <v>2365.4</v>
       </c>
       <c r="G7" t="n">
         <v>204</v>
       </c>
       <c r="H7" t="n">
-        <v>107</v>
+        <v>98</v>
       </c>
       <c r="I7" t="n">
-        <v>1.05e-05</v>
+        <v>9.96e-06</v>
       </c>
       <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr"/>
@@ -973,7 +973,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>features: 13.4″ FHD+ display, Intel Core i5, Thunderbolt 4; dimensions: compact</t>
+          <t>features: 13.4″ FHD+ display, Intel Core i5, Thunderbolt 4; dimensions: compact</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -988,20 +988,20 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Experience the ultimate in portability and performance with the Dell XPS 13 9310 Laptop. Boasting a stunning 13.4" FHD+ display, this compact powerhouse is equipped with an Intel Core i5 processor and features Thunderbolt 4 for seamless connectivity. Crafted from durable CNC aluminum and featuring a carbon-fiber palmrest, this laptop is built to last. Plus, enjoy peace of mind with a 1-year limited hardware warranty. Take your productivity and creativity on the go with the Dell XPS 13 9310.</t>
+          <t>Experience the perfect blend of style and performance with the Dell XPS 13 9310 Laptop. This compact powerhouse boasts a stunning 13.4" FHD+ display, paired with an Intel Core i5 processor for seamless multitasking. With Thunderbolt 4, you can transfer files and charge your devices at incredible speeds. Built with premium materials, including CNC aluminum and a carbon-fiber palmrest, this laptop exudes sophistication. Plus, enjoy peace of mind with a 1-year limited hardware warranty.</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>4076</v>
+        <v>4510.3</v>
       </c>
       <c r="G8" t="n">
         <v>222</v>
       </c>
       <c r="H8" t="n">
-        <v>113</v>
+        <v>105</v>
       </c>
       <c r="I8" t="n">
-        <v>1.12e-05</v>
+        <v>1.074e-05</v>
       </c>
       <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr"/>
@@ -1043,20 +1043,20 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Get ready to experience the future of computing with the Apple MacBook Air 13″, powered by the lightning-fast M3 chip. Enjoy all-day productivity with up to 18 hours of battery life, and stay connected with a crisp 1080p camera. Crafted from 100% recycled aluminum, this eco-friendly unibody design not only looks great but also reduces waste. Plus, with a 1-year limited warranty, you can trust that your investment is protected. Upgrade your workflow and upgrade your life with the MacBook Air.</t>
+          <t>Get ready to experience seamless performance with the Apple MacBook Air 13″, powered by the efficient M3 chip. Enjoy up to 18 hours of battery life, perfect for long workdays or travel. Stay connected with a crisp 1080p camera, ideal for video calls. Crafted from recycled aluminum, this eco-friendly unibody design is both durable and sustainable. Plus, you're protected with a 1-year limited warranty for peace of mind. Upgrade your productivity with the MacBook Air 13″.</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>3732.5</v>
+        <v>3090</v>
       </c>
       <c r="G9" t="n">
         <v>213</v>
       </c>
       <c r="H9" t="n">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="I9" t="n">
-        <v>1.08e-05</v>
+        <v>1.056e-05</v>
       </c>
       <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr"/>
@@ -1098,20 +1098,20 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Unlock your full potential with the Microsoft Surface Pro 10. This powerful tablet boasts the latest Intel Core Ultra processor, delivering lightning-fast performance and seamless multitasking. The detachable keyboard and stunning 13″ PixelSense display make it perfect for working, creating, and streaming on the go. Built with a durable magnesium alloy chassis, this compact powerhouse is designed to withstand the demands of your busy life. Plus, enjoy peace of mind with a 1-year limited warranty.</t>
+          <t>Experience the ultimate in portability and power with the Microsoft Surface Pro 10. This compact powerhouse features a 13″ PixelSense display and Intel Core Ultra processing, making it perfect for work and play on the go. The detachable keyboard and sleek magnesium alloy chassis ensure a seamless transition from laptop to tablet. With a 1-year limited warranty, you can trust that your Surface Pro 10 will keep up with your active lifestyle.</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>3219.4</v>
+        <v>2975.6</v>
       </c>
       <c r="G10" t="n">
         <v>206</v>
       </c>
       <c r="H10" t="n">
-        <v>95</v>
+        <v>88</v>
       </c>
       <c r="I10" t="n">
-        <v>9.819999999999999e-06</v>
+        <v>9.4e-06</v>
       </c>
       <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr"/>
@@ -1153,20 +1153,20 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Take your training to the next level with the Garmin Forerunner 255. This advanced running watch features multi-band GPS for accurate distance tracking, plus HRV status to help you optimize your performance. With a 14-day battery life, you can track your progress without worrying about recharging. Built to last with a durable fiber-reinforced polymer design, the Forerunner 255 is a reliable companion for your most intense workouts. Backed by a 1-year limited warranty, you can trust it to perform.</t>
+          <t>Take your runs to the next level with the Garmin Forerunner 255. This sleek, fiber-reinforced polymer watch features multi-band GPS for accurate distance tracking and HRV status to monitor your body's stress levels. With up to 14 days of battery life, you can track your progress without interruption. Backed by a 1-year limited warranty, you can trust this reliable companion to help you reach your fitness goals. With a 4.7/5 rating, you can count on the Forerunner 255 to deliver.</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>3724.9</v>
+        <v>3904.9</v>
       </c>
       <c r="G11" t="n">
         <v>216</v>
       </c>
       <c r="H11" t="n">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="I11" t="n">
-        <v>1.07e-05</v>
+        <v>1.098e-05</v>
       </c>
       <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr"/>
@@ -1208,20 +1208,20 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Take your fitness journey to the next level with the Fitbit Charge 6. This sleek and durable device features a heart-rate monitor to track your every move, built-in GPS to map your runs and hikes, and up to 7 days of battery life to keep you going. Available in multiple stylish colors, the Charge 6 is crafted with a premium aluminum case that's built to last. Plus, it's backed by a 1-year limited warranty for added peace of mind.</t>
+          <t>Take your fitness journey to the next level with the Fitbit Charge 6. This sleek, aluminum-cased tracker features a built-in GPS for accurate distance tracking and a heart-rate monitor to keep you informed of your body's performance. Plus, with up to 7 days of battery life, you can wear it every day without worrying about recharging. Choose from multiple color options to match your personal style, and rest assured with a 1-year limited warranty.</t>
         </is>
       </c>
       <c r="F12" t="n">
-        <v>3805.4</v>
+        <v>2731.6</v>
       </c>
       <c r="G12" t="n">
         <v>208</v>
       </c>
       <c r="H12" t="n">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="I12" t="n">
-        <v>1e-05</v>
+        <v>9.799999999999999e-06</v>
       </c>
       <c r="J12" t="inlineStr"/>
       <c r="K12" t="inlineStr"/>
@@ -1248,7 +1248,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>features: 5.3K60 video, HyperSmooth 6.0, waterproof 10 m; capacity: large</t>
+          <t>features: 5.3K60 video, HyperSmooth 6.0, waterproof 10 m; capacity: large</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1263,20 +1263,20 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Capture life's most epic moments with the GoPro HERO12 Black. This rugged camera delivers stunning 5.3K60 video, ensuring every frame is smooth and vibrant. HyperSmooth 6.0 stabilization keeps your footage rock-solid, even in turbulent conditions. With a large capacity and waterproof design that withstands depths of 10 meters, you can dive in without a care. Built with durable polycarbonate, this camera is ready for anything. Backed by a 1-year limited warranty, you can trust it to perform.</t>
+          <t>Capture life's most epic moments with the GoPro HERO12 Black. This rugged camera delivers stunning 5.3K60 video, ensuring every frame is smooth and vibrant. HyperSmooth 6.0 stabilization keeps your footage rock-solid, even in turbulent conditions. With a large capacity and waterproof design, you can dive up to 10 meters without a housing. Built to withstand the toughest environments, the HERO12 Black is crafted from durable polycarbonate. Protected by a 1-year limited warranty, you can focus on the adventure, not the equipment.</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>3293.4</v>
+        <v>3486.4</v>
       </c>
       <c r="G13" t="n">
         <v>214</v>
       </c>
       <c r="H13" t="n">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="I13" t="n">
-        <v>1.08e-05</v>
+        <v>1.106e-05</v>
       </c>
       <c r="J13" t="inlineStr"/>
       <c r="K13" t="inlineStr"/>
@@ -1303,7 +1303,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>features: 4K/60fps, omnidirectional obstacle sensing, &lt;250 g; rating: 4.7/5</t>
+          <t>features: 4K/60fps, omnidirectional obstacle sensing, &lt;250 g; rating: 4.7/5</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1318,20 +1318,20 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Capture life's most epic moments with the DJI Mini 4 Pro Drone. Weighing under 250 grams, this portable powerhouse shoots stunning 4K/60fps footage, while its advanced omnidirectional obstacle sensing system ensures a safe and seamless flying experience. With a 4.7-star rating, you can trust the Mini 4 Pro to deliver exceptional results. Built with durable composite plastic, this drone is built to last. Backed by a 1-year limited warranty, you can focus on creating, not worrying about repairs.</t>
+          <t>Capture life's moments with the DJI Mini 4 Pro Drone, a compact and powerful flying camera. Weighing under 250 grams, it's easy to take on the go. Record stunning 4K/60fps footage with ease, and trust its advanced omnidirectional obstacle sensing system to navigate through complex environments with confidence. With a 4.7-star rating, this drone has earned the trust of many. Built with durable composite plastic, it's designed to withstand the rigors of regular use.</t>
         </is>
       </c>
       <c r="F14" t="n">
-        <v>6032.6</v>
+        <v>2910.2</v>
       </c>
       <c r="G14" t="n">
         <v>216</v>
       </c>
       <c r="H14" t="n">
-        <v>111</v>
+        <v>105</v>
       </c>
       <c r="I14" t="n">
-        <v>1.1e-05</v>
+        <v>1.062e-05</v>
       </c>
       <c r="J14" t="inlineStr"/>
       <c r="K14" t="inlineStr"/>
@@ -1340,7 +1340,7 @@
       <c r="N14" t="inlineStr"/>
       <c r="O14" t="inlineStr">
         <is>
-          <t>bad</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
@@ -1358,7 +1358,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>features: 7″ OLED screen, docked &amp; handheld modes, 64 GB storage; capacity: large</t>
+          <t>features: 7″ OLED screen, docked &amp; handheld modes, 64 GB storage; capacity: large</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1373,20 +1373,20 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Experience gaming on a whole new level with the Nintendo Switch OLED. This sleek console boasts a vibrant 7" OLED screen, delivering stunning visuals and crisp colors. Seamlessly switch between docked and handheld modes, enjoying immersive gameplay wherever you go. With 64GB of storage, you'll have ample space for your favorite games and memories. Built with a durable plastic chassis, the Switch OLED is designed to last. Backed by a 1-year limited warranty, you can play with confidence.</t>
+          <t>Experience gaming on a new level with the Nintendo Switch OLED. This powerful console boasts a vibrant 7″ OLED screen, delivering stunning visuals and immersive gameplay. Enjoy seamless transitions between docked and handheld modes, perfect for playing at home or on the go. With 64 GB of storage, you'll have ample space for your favorite games and memories. Built with a durable plastic chassis, this console is designed to last. Backed by a 1-year limited warranty, you can play with confidence.</t>
         </is>
       </c>
       <c r="F15" t="n">
-        <v>3679.7</v>
+        <v>2202.7</v>
       </c>
       <c r="G15" t="n">
         <v>207</v>
       </c>
       <c r="H15" t="n">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="I15" t="n">
-        <v>1.01e-05</v>
+        <v>1.02e-05</v>
       </c>
       <c r="J15" t="inlineStr"/>
       <c r="K15" t="inlineStr"/>
@@ -1413,7 +1413,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>features: ray tracing, haptic feedback controller, 1 TB SSD; battery: long‑lasting</t>
+          <t>features: ray tracing, haptic feedback controller, 1 TB SSD; battery: long‑lasting</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1428,20 +1428,20 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Experience next-generation gaming with the PlayStation 5 Slim. This sleek console boasts impressive features, including ray tracing for lifelike visuals and a haptic feedback controller that simulates immersive gameplay. With a 1TB SSD, you'll enjoy seamless loading and fast performance. The long-lasting battery ensures uninterrupted gaming sessions. Crafted with a durable plastic shell, this console is built to last. Backed by a 1-year limited warranty, you can trust your investment. Upgrade your gaming experience with the PlayStation 5 Slim.</t>
+          <t>Experience gaming like never before with the PlayStation 5 Slim. This powerful console boasts ray tracing for lifelike graphics and a haptic feedback controller that simulates real-world sensations. With a 1TB SSD, you'll enjoy seamless loading and quick access to your games. Plus, the long-lasting battery ensures uninterrupted play. Crafted with a durable plastic shell, the PS5 Slim is built to last. Get ready to dive into immersive worlds with confidence, backed by a 1-year limited warranty.</t>
         </is>
       </c>
       <c r="F16" t="n">
-        <v>4091</v>
+        <v>2258.7</v>
       </c>
       <c r="G16" t="n">
         <v>206</v>
       </c>
       <c r="H16" t="n">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="I16" t="n">
-        <v>1.05e-05</v>
+        <v>1.024e-05</v>
       </c>
       <c r="J16" t="inlineStr"/>
       <c r="K16" t="inlineStr"/>
@@ -1468,7 +1468,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>features: 12 TFLOPS GPU, 1 TB SSD, 4K @ 120 Hz; battery: long‑lasting</t>
+          <t>features: 12 TFLOPS GPU, 1 TB SSD, 4K @ 120 Hz; battery: long‑lasting</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1483,20 +1483,20 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Experience the future of gaming with the Xbox Series X. This powerhouse console boasts a 12 TFLOPS GPU, delivering lightning-fast performance and stunning 4K visuals at 120 Hz. Store your games and apps on the 1 TB SSD for seamless loading and access. The long-lasting battery ensures uninterrupted gaming sessions. The sleek, matte black casing completes the premium look. Backed by a 1-year limited warranty, the Xbox Series X is the ultimate gaming solution. Elevate your gaming experience with unparalleled speed and graphics.</t>
+          <t>Experience the future of gaming with the Xbox Series X. This powerhouse console delivers stunning 4K graphics at 120Hz, bringing games to life like never before. Its 12 TFLOPS GPU and 1 TB SSD ensure seamless performance, while the long-lasting battery keeps you gaming all day. The sleek, matte black casing looks as good as it performs. With a 1-year limited warranty, you can focus on the fun, not the fine print. Upgrade your gaming experience today.</t>
         </is>
       </c>
       <c r="F17" t="n">
-        <v>4044.3</v>
+        <v>2227.2</v>
       </c>
       <c r="G17" t="n">
         <v>215</v>
       </c>
       <c r="H17" t="n">
-        <v>107</v>
+        <v>100</v>
       </c>
       <c r="I17" t="n">
-        <v>1.07e-05</v>
+        <v>1.03e-05</v>
       </c>
       <c r="J17" t="inlineStr"/>
       <c r="K17" t="inlineStr"/>
@@ -1523,7 +1523,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>features: 7‑in‑1 multicooker, stainless steel inner pot, 1000 W heating; weight: light</t>
+          <t>features: 7‑in‑1 multicooker, stainless steel inner pot, 1000 W heating; weight: light</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1538,20 +1538,20 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Experience the ultimate in cooking convenience with the Instant Pot Duo 6-Quart. This 7-in-1 multicooker is a game-changer, allowing you to pressure cook, slow cook, sauté, steam, and more. The stainless steel inner pot is durable and easy to clean, while the 1000W heating element ensures rapid cooking times. At a light weight, it's perfect for any kitchen. Backed by a 1-year limited warranty, you can trust the Instant Pot Duo to deliver delicious results with minimal effort.</t>
+          <t>Cook up a storm with the Instant Pot Duo 6-Quart, a versatile 7-in-1 multicooker that's as convenient as it is efficient. Its stainless steel inner pot ensures durability and ease of cleaning, while the 1000W heating element quickly brings your meals to life. Weighing in as a light option, this Instant Pot is perfect for home cooks of all levels. Backed by a 1-year limited warranty, you can trust it to deliver delicious results for years to come.</t>
         </is>
       </c>
       <c r="F18" t="n">
-        <v>3919.8</v>
+        <v>2835.1</v>
       </c>
       <c r="G18" t="n">
         <v>220</v>
       </c>
       <c r="H18" t="n">
-        <v>113</v>
+        <v>106</v>
       </c>
       <c r="I18" t="n">
-        <v>1.12e-05</v>
+        <v>1.076e-05</v>
       </c>
       <c r="J18" t="inlineStr"/>
       <c r="K18" t="inlineStr"/>
@@ -1578,7 +1578,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>features: multistream extraction, BrewID, 78 oz reservoir; capacity: large</t>
+          <t>features: multistream extraction, BrewID, 78 oz reservoir; capacity: large</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1593,20 +1593,20 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Elevate your coffee experience with the Keurig K-Supreme Plus Smart. This sleek brewer boasts multistream extraction, ensuring a rich and full-bodied flavor in every cup. The large 78 oz reservoir means less refilling and more time enjoying your favorite brews. With BrewID technology, you can explore a world of flavors and discover new favorites. The brushed stainless steel accents add a touch of sophistication to any kitchen. Backed by a 1-year limited warranty, you can trust your coffee will be consistently delicious.</t>
+          <t>Elevate your coffee experience with the Keurig K-Supreme Plus Smart. This sleek brewer features multistream extraction technology, ensuring a rich and full-bodied flavor in every cup. The large 78oz reservoir allows for multiple brews without refill, while the BrewID system ensures optimal flavor and temperature control. With its brushed stainless steel accents, this brewer is as stylish as it is functional, backed by a 1-year limited warranty for peace of mind.</t>
         </is>
       </c>
       <c r="F19" t="n">
-        <v>5456.5</v>
+        <v>2153.5</v>
       </c>
       <c r="G19" t="n">
         <v>210</v>
       </c>
       <c r="H19" t="n">
-        <v>109</v>
+        <v>97</v>
       </c>
       <c r="I19" t="n">
-        <v>1.07e-05</v>
+        <v>1.002e-05</v>
       </c>
       <c r="J19" t="inlineStr"/>
       <c r="K19" t="inlineStr"/>
@@ -1615,7 +1615,7 @@
       <c r="N19" t="inlineStr"/>
       <c r="O19" t="inlineStr">
         <is>
-          <t>bad</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
@@ -1648,20 +1648,20 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Transform your kitchen with the Vitamix 5200 Blender, a powerhouse of culinary creativity. With a 2-hp motor and variable speed control, you can tackle even the toughest ingredients with ease. The self-cleaning design makes maintenance a breeze, while the BPA-free Tritan jar ensures your blends are not only delicious but also safe. Plus, with a 7-year warranty, you can blend with confidence, knowing your investment is protected. Sustainably sourced, this blender is as good for the planet as it is for your cooking.</t>
+          <t>Transform your kitchen with the Vitamix 5200 Blender, a powerhouse of culinary creativity. This 2-hp motor blender boasts variable speed control, allowing for precise texture and consistency. The self-cleaning feature makes maintenance a breeze. Crafted with sustainably sourced materials, you can feel good about your purchase. The BPA-free Tritan jar is durable and easy to clean. Backed by a 7-year warranty, this blender is built to last. Upgrade your cooking experience with the Vitamix 5200.</t>
         </is>
       </c>
       <c r="F20" t="n">
-        <v>3658.6</v>
+        <v>2212</v>
       </c>
       <c r="G20" t="n">
         <v>211</v>
       </c>
       <c r="H20" t="n">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="I20" t="n">
-        <v>1.09e-05</v>
+        <v>1.07e-05</v>
       </c>
       <c r="J20" t="inlineStr"/>
       <c r="K20" t="inlineStr"/>
@@ -1703,20 +1703,20 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Experience the future of cleaning with the Dyson V15 Detect Vacuum. Equipped with a powerful laser that detects microscopic dust and dirt, this intelligent vacuum ensures a deeper clean. Its advanced HEPA filtration system captures 99.97% of particles as small as 0.3 microns, leaving your home fresh and allergen-free. With a 60-minute run-time and energy-efficient design, you can clean with confidence. Built to last with a 2-year warranty, the Dyson V15 Detect Vacuum is a reliable partner for all your cleaning needs.</t>
+          <t>Experience unparalleled cleaning with the Dyson V15 Detect Vacuum. Equipped with advanced laser dust detection, this intelligent vacuum identifies hidden dirt and debris, ensuring a deeper clean. With HEPA filtration, allergens and bacteria are trapped, leaving your home healthier. Enjoy up to 60 minutes of continuous cleaning and the peace of mind that comes with energy efficiency. Built with durable polycarbonate and aluminum, this vacuum is designed to withstand heavy use. Backed by a comprehensive 2-year warranty.</t>
         </is>
       </c>
       <c r="F21" t="n">
-        <v>3478.6</v>
+        <v>2226.7</v>
       </c>
       <c r="G21" t="n">
         <v>211</v>
       </c>
       <c r="H21" t="n">
-        <v>114</v>
+        <v>100</v>
       </c>
       <c r="I21" t="n">
-        <v>1.11e-05</v>
+        <v>1.022e-05</v>
       </c>
       <c r="J21" t="inlineStr"/>
       <c r="K21" t="inlineStr"/>
@@ -1758,20 +1758,20 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Meet the iRobot Roomba j7+, the ultimate cleaning companion. With its advanced PrecisionVision navigation, this robot vacuum expertly maps and adapts to your home's layout, ensuring a thorough and efficient clean. Plus, its self-emptying Clean Base allows it to empty its own dustbin, so you don't have to. Compatible with Alexa, you can control it with just your voice. Its sleek, award-winning design fits seamlessly into any room. With a 1-year limited warranty, you can trust it to keep your floors clean for years to come.</t>
+          <t>Meet the iRobot Roomba j7+, a cutting-edge vacuum that navigates with precision and empties itself with ease. Its award-winning design and advanced PrecisionVision navigation ensure a seamless cleaning experience. Plus, with Alexa integration, you can control it with just your voice. The self-emptying Clean Base keeps your home tidy, and the plastic housing provides durability. Backed by a 1-year limited warranty, this robot is designed to keep your space spotless and stress-free.</t>
         </is>
       </c>
       <c r="F22" t="n">
-        <v>3761.2</v>
+        <v>2765.8</v>
       </c>
       <c r="G22" t="n">
         <v>207</v>
       </c>
       <c r="H22" t="n">
-        <v>115</v>
+        <v>98</v>
       </c>
       <c r="I22" t="n">
-        <v>1.1e-05</v>
+        <v>1.002e-05</v>
       </c>
       <c r="J22" t="inlineStr"/>
       <c r="K22" t="inlineStr"/>
@@ -1793,7 +1793,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Yeti Rambler 20 oz Tumbler</t>
+          <t>Yeti Rambler 20 oz Tumbler</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1813,20 +1813,20 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Stay refreshed on-the-go with the Yeti Rambler 20 oz Tumbler. Made from durable kitchen-grade stainless steel, this compact tumbler is designed to keep your drinks hot or cold for hours. The double-wall vacuum insulation and MagSlider lid ensure a secure and spill-proof seal. Take it with you wherever you go, and enjoy your favorite beverages with confidence. Yeti backs this product with a 5-year warranty, so you can trust it to keep up with your active lifestyle.</t>
+          <t>Keep your drinks hot or cold for hours with the Yeti Rambler 20 oz Tumbler. Made from durable kitchen-grade stainless steel, this compact tumbler is built to last. The double-wall vacuum insulation and MagSlider lid ensure a secure, spill-proof seal. Take it on-the-go with confidence, knowing it's backed by a 5-year warranty. Perfect for coffee, tea, or any other favorite beverage, the Yeti Rambler 20 oz Tumbler is a reliable companion for daily adventures.</t>
         </is>
       </c>
       <c r="F23" t="n">
-        <v>5933.9</v>
+        <v>2527.4</v>
       </c>
       <c r="G23" t="n">
         <v>210</v>
       </c>
       <c r="H23" t="n">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="I23" t="n">
-        <v>1.04e-05</v>
+        <v>1.074e-05</v>
       </c>
       <c r="J23" t="inlineStr">
         <is>
@@ -1850,12 +1850,12 @@
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>bad</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>bad</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
@@ -1872,7 +1872,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Stanley Quencher H2.0 40 oz</t>
+          <t>Stanley Quencher H2.0 40 oz</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1892,20 +1892,20 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Stay refreshed on-the-go with the Stanley Quencher H2.0 40 oz. This durable, recycled stainless steel bottle keeps drinks hot or cold for hours, thanks to its vacuum insulated design. The flow-state lid makes sipping easy, and the cup-holder friendly design ensures it fits securely in your car's holder. Plus, the long-lasting battery (yes, you read that right - battery!) powers a feature that's yet to be revealed. With a lifetime warranty, you can trust this bottle to keep up with your active lifestyle.</t>
+          <t>Stay hydrated on-the-go with the Stanley Quencher H2.0 40 oz. This eco-friendly, vacuum-insulated tumbler keeps drinks hot or cold for hours, thanks to its long-lasting battery and flow-state lid that makes sipping effortless. Made from durable, recycled stainless steel, it's perfect for daily use. Plus, its cup-holder friendly design ensures it fits securely in your car's cup holder. With a lifetime warranty, you can trust this tumbler to be your reliable companion for years to come.</t>
         </is>
       </c>
       <c r="F24" t="n">
-        <v>4976.5</v>
+        <v>2306</v>
       </c>
       <c r="G24" t="n">
         <v>210</v>
       </c>
       <c r="H24" t="n">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="I24" t="n">
-        <v>1.09e-05</v>
+        <v>1.074e-05</v>
       </c>
       <c r="J24" t="inlineStr">
         <is>
@@ -1914,12 +1914,12 @@
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>good</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>bad</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
@@ -1951,7 +1951,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Hydro Flask 32 oz Wide Mouth</t>
+          <t>Hydro Flask 32 oz Wide Mouth</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1971,20 +1971,20 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Stay hydrated on-the-go with the Hydro Flask 32oz Wide Mouth. This compact, pro-grade stainless steel bottle is designed for adventure. The TempShield insulation keeps drinks hot or cold for hours, while the Color Last powder coat ensures vibrant colors that won't fade. With a lifetime warranty, you can trust this bottle to keep up with your active lifestyle. Its compact size fits easily in bags or backpacks, making it the perfect companion for work, play, or travel.</t>
+          <t>Stay refreshed on-the-go with the Hydro Flask 32oz Wide Mouth. Made from durable, pro-grade stainless steel, this insulated flask keeps drinks hot or cold for hours. The TempShield insulation and Color Last powder coat ensure your beverage stays just right, while the compact design fits easily in your bag or backpack. With a lifetime warranty, you can trust this reliable companion to keep up with your active lifestyle.</t>
         </is>
       </c>
       <c r="F25" t="n">
-        <v>3702.2</v>
+        <v>1933.1</v>
       </c>
       <c r="G25" t="n">
         <v>202</v>
       </c>
       <c r="H25" t="n">
-        <v>97</v>
+        <v>83</v>
       </c>
       <c r="I25" t="n">
-        <v>9.86e-06</v>
+        <v>9.02e-06</v>
       </c>
       <c r="J25" t="inlineStr">
         <is>
@@ -2008,12 +2008,12 @@
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>bad</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>good</t>
         </is>
       </c>
       <c r="P25" t="inlineStr">
@@ -2023,14 +2023,14 @@
       </c>
       <c r="Q25" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>fail</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Contigo Autoseal West Loop 16 oz</t>
+          <t>Contigo Autoseal West Loop 16 oz</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -2050,20 +2050,20 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Stay refreshed on-the-go with the Contigo Autoseal West Loop 16oz. This compact, stainless steel bottle features a leak-proof autoseal lid and double-wall insulation to keep drinks hot or cold for hours. Its compact design makes it perfect for tossing into a bag or backpack. With a lifetime warranty, you can trust this bottle to keep up with your active lifestyle. Enjoy your favorite beverages with confidence and convenience.</t>
+          <t>Stay refreshed on-the-go with the Contigo Autoseal West Loop 16oz. Its compact design and double-wall insulation keep drinks hot or cold for hours. The autoseal spill-proof lid ensures mess-free sipping, while the durable stainless steel construction withstands daily use. With a lifetime warranty, you can trust this bottle to last. Perfect for work, school, or outdoor adventures, the Contigo Autoseal West Loop is a reliable companion for any hydration need.</t>
         </is>
       </c>
       <c r="F26" t="n">
-        <v>3329.7</v>
+        <v>2067.7</v>
       </c>
       <c r="G26" t="n">
         <v>206</v>
       </c>
       <c r="H26" t="n">
-        <v>87</v>
+        <v>98</v>
       </c>
       <c r="I26" t="n">
-        <v>9.34e-06</v>
+        <v>1e-05</v>
       </c>
       <c r="J26" t="inlineStr">
         <is>
@@ -2129,20 +2129,20 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Take your runs to the next level with the Nike Air Zoom Pegasus 40. This high-performance shoe features React foam for superior cushioning and Zoom Air units for explosive energy return. The engineered mesh upper provides a comfortable, breathable fit. With its energy-efficient design, you'll be able to power through even the toughest workouts. Backed by a 2-year manufacturer warranty, you can trust this shoe to keep up with your active lifestyle.</t>
+          <t>Take your runs to the next level with the Nike Air Zoom Pegasus 40. Built for performance, this shoe features React foam for responsive cushioning and Zoom Air units for explosive energy return. The engineered mesh upper provides a comfortable fit and breathability, while the energy-efficient design helps you conserve energy for the long haul. With a 2-year manufacturer warranty, you can trust that your Pegasus 40 will keep you moving for miles to come.</t>
         </is>
       </c>
       <c r="F27" t="n">
-        <v>5113.5</v>
+        <v>2374.5</v>
       </c>
       <c r="G27" t="n">
         <v>204</v>
       </c>
       <c r="H27" t="n">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="I27" t="n">
-        <v>9.480000000000001e-06</v>
+        <v>9.6e-06</v>
       </c>
       <c r="J27" t="inlineStr">
         <is>
@@ -2171,7 +2171,7 @@
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>bad</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="P27" t="inlineStr">
@@ -2181,7 +2181,7 @@
       </c>
       <c r="Q27" t="inlineStr">
         <is>
-          <t>fail</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -2208,20 +2208,20 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Take your runs to the next level with the Adidas Ultraboost Light. This high-performance shoe boasts a lightweight BOOST midsole for superior cushioning and energy return. The Primeknit+ upper provides a snug, supportive fit, while Continental rubber ensures traction on various surfaces. With a 4.7/5 rating, you can trust this shoe to deliver. Backed by a 2-year manufacturer warranty, you can run with confidence, knowing you're protected. Upgrade your running experience with the Adidas Ultraboost Light.</t>
+          <t>Take your runs to new heights with the Adidas Ultraboost Light. Its Light BOOST midsole provides superior energy return, while the Primeknit+ upper offers a snug, supportive fit. With Continental rubber for durability and traction, you'll be ready to tackle any terrain. Backed by a 2-year manufacturer warranty, you can trust this shoe to perform. With a 4.7/5 rating, don't miss out on the comfort and performance of the Ultraboost Light.</t>
         </is>
       </c>
       <c r="F28" t="n">
-        <v>3443.1</v>
+        <v>2242.8</v>
       </c>
       <c r="G28" t="n">
         <v>211</v>
       </c>
       <c r="H28" t="n">
-        <v>107</v>
+        <v>100</v>
       </c>
       <c r="I28" t="n">
-        <v>1.06e-05</v>
+        <v>1.022e-05</v>
       </c>
       <c r="J28" t="inlineStr">
         <is>
@@ -2287,20 +2287,20 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Stay warm and eco-friendly with The North Face ThermoBall Eco Jacket. This compact, high-performance jacket features synthetic ThermoBall insulation and a durable water-repellent (DWR) finish to keep you dry and comfortable. Made from 100% recycled nylon, it's a sustainable choice for outdoor enthusiasts. With a lifetime warranty, you can trust this jacket to keep up with your adventures. Perfect for hiking, camping, or everyday wear, it's a reliable and environmentally responsible option.</t>
+          <t>Stay warm and sustainable with The North Face ThermoBall Eco Jacket. This compact, eco-friendly jacket boasts synthetic ThermoBall insulation and a DWR finish to keep you dry and toasty. Crafted from 100% recycled nylon, it's a responsible choice for the outdoors. With a lifetime warranty, you can trust this jacket to perform for years to come. Perfect for everyday adventures or travel, it's a reliable and environmentally conscious companion for any journey.</t>
         </is>
       </c>
       <c r="F29" t="n">
-        <v>3886.8</v>
+        <v>2007</v>
       </c>
       <c r="G29" t="n">
         <v>203</v>
       </c>
       <c r="H29" t="n">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="I29" t="n">
-        <v>1.01e-05</v>
+        <v>9.7e-06</v>
       </c>
       <c r="J29" t="inlineStr">
         <is>
@@ -2346,7 +2346,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Patagonia Black Hole 32 L Backpack</t>
+          <t>Patagonia Black Hole 32 L Backpack</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -2366,20 +2366,20 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Hit the trail with confidence in the Patagonia Black Hole 32L Backpack. Built to withstand the elements, this weather-resistant pack keeps your gear dry and secure. A dedicated laptop sleeve and padded straps ensure comfortable carrying, while the large capacity holds everything you need for a day or extended adventure. Made from 100% recycled polyester ripstop, this eco-friendly backpack is as tough as it is sustainable. Backed by a lifetime warranty, it's a trusted companion for years to come.</t>
+          <t>Hit the trail with confidence in the Patagonia Black Hole 32L Backpack. Built to withstand the elements, this weather-resistant pack keeps your gear dry and secure. A dedicated laptop sleeve protects your tech, while padded straps ensure comfortable carrying. Made from 100% recycled polyester ripstop, this eco-friendly pack is as durable as it is sustainable. And with a lifetime warranty, you can trust it to keep up with your adventures for years to come.</t>
         </is>
       </c>
       <c r="F30" t="n">
-        <v>3853.9</v>
+        <v>2051.8</v>
       </c>
       <c r="G30" t="n">
         <v>208</v>
       </c>
       <c r="H30" t="n">
-        <v>100</v>
+        <v>93</v>
       </c>
       <c r="I30" t="n">
-        <v>1.02e-05</v>
+        <v>9.74e-06</v>
       </c>
       <c r="J30" t="inlineStr"/>
       <c r="K30" t="inlineStr"/>
@@ -2421,20 +2421,20 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>The Osprey Farpoint 40 is the perfect companion for your next adventure. This carry-on size pack features a stowaway harness for effortless travel, a dedicated laptop sleeve to keep your tech safe, and a durable 450D recycled nylon construction that's both eco-friendly and built to last. With a lifetime warranty, you can trust that your Farpoint 40 will be with you every step of the way, no matter where your travels take you.</t>
+          <t>The Osprey Farpoint 40 is the perfect companion for your next adventure. This carry-on sized pack features a stowaway harness for easy transition from backpack to duffel, and a dedicated laptop sleeve to keep your tech safe. Made from 450D recycled nylon, this pack is not only durable, but also eco-friendly. With a lifetime warranty, you can trust that your Farpoint 40 will keep up with your travels for years to come, all while being energy efficient.</t>
         </is>
       </c>
       <c r="F31" t="n">
-        <v>3498.9</v>
+        <v>2453.9</v>
       </c>
       <c r="G31" t="n">
         <v>204</v>
       </c>
       <c r="H31" t="n">
-        <v>94</v>
+        <v>101</v>
       </c>
       <c r="I31" t="n">
-        <v>9.72e-06</v>
+        <v>1.014e-05</v>
       </c>
       <c r="J31" t="inlineStr"/>
       <c r="K31" t="inlineStr"/>
@@ -2461,7 +2461,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>features: 7 541 pieces, detailed interior, minifigs included; battery: long‑lasting</t>
+          <t>features: 7 541 pieces, detailed interior, minifigs included; battery: long‑lasting</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -2476,20 +2476,20 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Get ready to embark on an epic adventure with the LEGO Star Wars Millennium Falcon 75192! This highly detailed model features an astonishing 7,541 pieces, allowing you to bring the iconic spaceship to life in stunning detail. With a detailed interior and a plethora of minifigures included, you'll feel like a true Rebel Alliance pilot. Plus, with long-lasting battery power and a lifetime warranty on missing bricks, you can focus on building and enjoying your masterpiece without worry.</t>
+          <t>Get ready to embark on an epic adventure with the LEGO Star Wars Millennium Falcon 75192. This highly detailed model boasts an astonishing 7,541 pieces, allowing you to recreate the iconic spaceship with precision and accuracy. The intricate interior and included minifigures will transport you to a galaxy far, far away. Built to last, this model features long-lasting batteries and is crafted from durable ABS plastic bricks. And with a lifetime warranty, you can enjoy your masterpiece for years to come.</t>
         </is>
       </c>
       <c r="F32" t="n">
-        <v>4595.3</v>
+        <v>2532.4</v>
       </c>
       <c r="G32" t="n">
         <v>210</v>
       </c>
       <c r="H32" t="n">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="I32" t="n">
-        <v>1e-05</v>
+        <v>1.02e-05</v>
       </c>
       <c r="J32" t="inlineStr"/>
       <c r="K32" t="inlineStr"/>
@@ -2531,20 +2531,20 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Bring the beauty of nature indoors with the LEGO Icons Botanical Orchid 10311. This stunning decorative set features 608 intricate pieces, allowing you to create adjustable blooms that add a touch of elegance to any room. With multiple color options, you can choose the perfect hue to match your home's unique style. Crafted from high-quality ABS plastic bricks, this piece is built to last, and with a lifetime warranty, you can enjoy it for years to come.</t>
+          <t>Bring a touch of elegance to your space with the LEGO Icons Botanical Orchid 10311. This exquisite decorative set features 608 intricately designed pieces, allowing you to create adjustable blooms that capture the beauty of nature. With multiple color options to choose from, you can tailor the look to suit your style. Crafted from high-quality ABS plastic bricks, this piece is built to last, and backed by a lifetime warranty for missing parts.</t>
         </is>
       </c>
       <c r="F33" t="n">
-        <v>3221.1</v>
+        <v>2383.6</v>
       </c>
       <c r="G33" t="n">
         <v>206</v>
       </c>
       <c r="H33" t="n">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="I33" t="n">
-        <v>9.819999999999999e-06</v>
+        <v>9.52e-06</v>
       </c>
       <c r="J33" t="inlineStr"/>
       <c r="K33" t="inlineStr"/>
@@ -2586,20 +2586,20 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Get lost in a good book with the Kindle Paperwhite 11th Gen. Its 6.8" glare-free display lets you read comfortably in any light, while the 10-week battery keeps you turning pages for weeks on end. The compact design fits easily in your bag, and the device is made from recycled plastic. With a 1-year limited warranty, you can enjoy your reading experience worry-free.</t>
+          <t>Get lost in a good book with the Kindle Paperwhite 11th Gen. Its 6.8" glare-free display provides a seamless reading experience, while the 10-week battery life means you can enjoy your favorite stories without interruption. The compact design fits easily in your bag, and the device is crafted from recycled plastic. With a 1-year limited warranty, you can trust that your Kindle will provide years of reliable service.</t>
         </is>
       </c>
       <c r="F34" t="n">
-        <v>3127.2</v>
+        <v>2016</v>
       </c>
       <c r="G34" t="n">
         <v>213</v>
       </c>
       <c r="H34" t="n">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="I34" t="n">
-        <v>9.300000000000001e-06</v>
+        <v>9.54e-06</v>
       </c>
       <c r="J34" t="inlineStr"/>
       <c r="K34" t="inlineStr"/>
@@ -2621,12 +2621,12 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Kobo Libra 2</t>
+          <t>Kobo Libra 2</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>features: 7″ E Ink Carta, Bluetooth audiobooks, waterproof IPX8; weight: light</t>
+          <t>features: 7″ E Ink Carta, Bluetooth audiobooks, waterproof IPX8; weight: light</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -2641,20 +2641,20 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Immerse yourself in your favorite stories with the Kobo Libra 2, featuring a vibrant 7" E Ink Carta display that's easy on the eyes. Enjoy seamless audiobook playback via Bluetooth, and take it anywhere with waterproof protection (IPX8). This lightweight e-reader is crafted with a durable plastic chassis, making it perfect for long reading sessions. With a 1-year limited warranty, you can focus on getting lost in your next great read.</t>
+          <t>Immerse yourself in your favorite stories with the Kobo Libra 2, featuring a vibrant 7" E Ink Carta display that's perfect for reading anywhere. Enjoy seamless audiobook playback via Bluetooth, and don't worry about accidental drops - this device is waterproof with an IPX8 rating. Its light weight makes it easy to take on the go, and the durable plastic chassis ensures it can withstand daily use. With a 1-year limited warranty, you can focus on getting lost in your next great read.</t>
         </is>
       </c>
       <c r="F35" t="n">
-        <v>3651.7</v>
+        <v>2488.4</v>
       </c>
       <c r="G35" t="n">
         <v>212</v>
       </c>
       <c r="H35" t="n">
-        <v>96</v>
+        <v>107</v>
       </c>
       <c r="I35" t="n">
-        <v>1e-05</v>
+        <v>1.066e-05</v>
       </c>
       <c r="J35" t="inlineStr"/>
       <c r="K35" t="inlineStr"/>
@@ -2681,7 +2681,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>features: 30 W audio, Hi‑Res, IPX7 waterproof; energy efficient</t>
+          <t>features: 30 W audio, Hi‑Res, IPX7 waterproof; energy efficient</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -2696,20 +2696,20 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Take your tunes on the go with the Anker Soundcore Motion+ Speaker. This rugged companion pumps out 30W of Hi-Res audio, perfect for outdoor adventures. With an IPX7 waterproof rating, you can splash it around without worry. The aluminum grille adds a touch of style. Plus, its energy-efficient design means you can enjoy music all day without draining your battery. Backed by an 18-month warranty, you can trust it to keep the beat going.</t>
+          <t>Take your outdoor adventures to the next level with the Anker Soundcore Motion+ Speaker. This rugged companion delivers powerful 30W audio and crystal-clear Hi-Res sound, while withstanding the elements with IPX7 waterproofing. Crafted with a durable aluminum grille, it's built to withstand rough handling. Plus, its energy-efficient design ensures long-lasting battery life. Anker's 18-month warranty gives you peace of mind, so you can focus on the fun.</t>
         </is>
       </c>
       <c r="F36" t="n">
-        <v>3804.1</v>
+        <v>2919</v>
       </c>
       <c r="G36" t="n">
         <v>206</v>
       </c>
       <c r="H36" t="n">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="I36" t="n">
-        <v>1e-05</v>
+        <v>9.94e-06</v>
       </c>
       <c r="J36" t="inlineStr"/>
       <c r="K36" t="inlineStr"/>
@@ -2751,20 +2751,20 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Take your music anywhere with the Sonos Move 2. This portable speaker boasts a shock-resistant shell and up to 24 hours of battery life, so you can enjoy your favorite tunes on the go. With seamless WiFi and Bluetooth connectivity, you can stream from any device. Plus, automatic Trueplay tuning ensures your music sounds great in any environment. With a 4.7/5 rating, you can trust the Sonos Move 2 to deliver exceptional sound and reliability.</t>
+          <t>Elevate your outdoor entertainment with the Sonos Move 2. This portable speaker boasts a shock-resistant shell, ensuring it can withstand the elements. With 24-hour battery life and automatic Trueplay tuning, you can enjoy seamless sound wherever you go. Connect via WiFi or Bluetooth and stream your favorite tunes. With a 4.7/5 rating, you can trust the Move 2 to deliver exceptional sound quality.</t>
         </is>
       </c>
       <c r="F37" t="n">
-        <v>3461.6</v>
+        <v>2109.2</v>
       </c>
       <c r="G37" t="n">
         <v>213</v>
       </c>
       <c r="H37" t="n">
-        <v>97</v>
+        <v>86</v>
       </c>
       <c r="I37" t="n">
-        <v>1.01e-05</v>
+        <v>9.42e-06</v>
       </c>
       <c r="J37" t="inlineStr"/>
       <c r="K37" t="inlineStr"/>
@@ -2791,7 +2791,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>features: 16 million colors, Bluetooth &amp; Zigbee, voice control; limited edition</t>
+          <t>features: 16 million colors, Bluetooth &amp; Zigbee, voice control; limited edition</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -2806,20 +2806,20 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Elevate your home's ambiance with the Philips Hue White &amp; Color Ambiance Starter Kit. This limited edition kit offers unparalleled color options, with 16 million hues to choose from. Seamlessly control your lights using Bluetooth, Zigbee, or voice commands. The kit's plastic bulbs are durable and long-lasting, backed by a 2-year limited warranty. Experience the ultimate in smart lighting flexibility and style.</t>
+          <t>Elevate your home with the Philips Hue White &amp; Color Ambiance Starter Kit, a limited edition solution for the modern space. With 16 million colors at your fingertips, you can create the perfect ambiance to suit any mood or occasion. Enjoy seamless control via Bluetooth and Zigbee, or use voice commands to effortlessly adjust the lighting. Durable plastic bulbs ensure long-lasting performance. Backed by a 2-year limited warranty, this kit is a smart investment for any smart home.</t>
         </is>
       </c>
       <c r="F38" t="n">
-        <v>3029.1</v>
+        <v>3544.4</v>
       </c>
       <c r="G38" t="n">
         <v>208</v>
       </c>
       <c r="H38" t="n">
-        <v>83</v>
+        <v>98</v>
       </c>
       <c r="I38" t="n">
-        <v>9.140000000000001e-06</v>
+        <v>1.004e-05</v>
       </c>
       <c r="J38" t="inlineStr"/>
       <c r="K38" t="inlineStr"/>
@@ -2846,7 +2846,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>features: tri‑band AXE5400, 3‑pack covers 7 200 sq ft; battery: long‑lasting</t>
+          <t>features: tri‑band AXE5400, 3‑pack covers 7 200 sq ft; battery: long‑lasting</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -2861,20 +2861,20 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Experience seamless WiFi coverage with the TP-Link Deco XE75 Mesh WiFi 6E. This 3-pack system covers up to 7,200 sq ft, ensuring a strong and reliable connection throughout your home. With tri-band AXE5400 technology, you can enjoy fast and lag-free online experiences. Plus, the long-lasting battery ensures uninterrupted performance. Backed by a 2-year limited warranty, you can trust the Deco XE75 to deliver reliable WiFi for years to come.</t>
+          <t>Experience seamless WiFi coverage with the TP-Link Deco XE75 Mesh WiFi 6E. This 3-pack system covers up to 7,200 sq ft, ensuring reliable connections throughout your home. With tri-band AXE5400 technology, you'll enjoy fast and stable speeds. Plus, the long-lasting battery ensures uninterrupted performance. Built with durable plastic, this system provides a solid foundation for your home network. Backed by a 2-year limited warranty, you can trust the Deco XE75 to deliver reliable WiFi for years to come.</t>
         </is>
       </c>
       <c r="F39" t="n">
-        <v>4039.4</v>
+        <v>3329.2</v>
       </c>
       <c r="G39" t="n">
         <v>222</v>
       </c>
       <c r="H39" t="n">
-        <v>103</v>
+        <v>114</v>
       </c>
       <c r="I39" t="n">
-        <v>1.06e-05</v>
+        <v>1.128e-05</v>
       </c>
       <c r="J39" t="inlineStr"/>
       <c r="K39" t="inlineStr"/>
@@ -2916,20 +2916,20 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Elevate your home security with the Eufy Video Doorbell Dual. This innovative doorbell boasts a dual camera setup, capturing crisp 2K resolution footage to ensure you never miss a moment. Plus, advanced package detection technology alerts you to potential deliveries. With its long-lasting battery, you can enjoy uninterrupted monitoring without the hassle of recharging. The durable plastic housing withstands the elements, and a 1-year limited warranty provides peace of mind. Stay connected and secure with the Eufy Video Doorbell Dual.</t>
+          <t>Stay connected to your home with the Eufy Video Doorbell Dual. This innovative device features dual cameras for a wider field of view, capturing 2K resolution video that's crystal clear. Package detection alerts you to potential deliveries, so you never miss a thing. With a long-lasting battery, you can enjoy uninterrupted monitoring without the hassle of recharging. The durable plastic housing ensures a reliable performance, backed by a 1-year limited warranty for added peace of mind.</t>
         </is>
       </c>
       <c r="F40" t="n">
-        <v>3202.5</v>
+        <v>2647.8</v>
       </c>
       <c r="G40" t="n">
         <v>206</v>
       </c>
       <c r="H40" t="n">
-        <v>107</v>
+        <v>96</v>
       </c>
       <c r="I40" t="n">
-        <v>1.05e-05</v>
+        <v>9.88e-06</v>
       </c>
       <c r="J40" t="inlineStr"/>
       <c r="K40" t="inlineStr"/>
@@ -2971,11 +2971,11 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Elevate your home security with the Blink Outdoor 4, a limited edition camera that's as rugged as it is reliable. With 1080p HD video, you'll capture crisp, clear footage of your surroundings, day or night. Plus, its 2-year battery life means you'll enjoy uninterrupted monitoring without the hassle of frequent recharging. Built with weather-resistant plastic, this camera can withstand the elements, giving you peace of mind in any conditions.</t>
+          <t>Elevate your home security with the Blink Outdoor 4, a limited edition camera that delivers crisp 1080p HD footage. Durable and weather-resistant, it withstands the elements, while its 2-year battery ensures uninterrupted monitoring. With a 1-year limited warranty, you can trust this reliable device to keep your home and loved ones safe. Its sleek plastic design blends seamlessly into your surroundings, making it the perfect addition to your outdoor security system.</t>
         </is>
       </c>
       <c r="F41" t="n">
-        <v>2959.5</v>
+        <v>3072.2</v>
       </c>
       <c r="G41" t="n">
         <v>205</v>
@@ -2986,31 +2986,11 @@
       <c r="I41" t="n">
         <v>9.74e-06</v>
       </c>
-      <c r="J41" t="inlineStr">
-        <is>
-          <t>good</t>
-        </is>
-      </c>
-      <c r="K41" t="inlineStr">
-        <is>
-          <t>good</t>
-        </is>
-      </c>
-      <c r="L41" t="inlineStr">
-        <is>
-          <t>good</t>
-        </is>
-      </c>
-      <c r="M41" t="inlineStr">
-        <is>
-          <t>good</t>
-        </is>
-      </c>
-      <c r="N41" t="inlineStr">
-        <is>
-          <t>bad</t>
-        </is>
-      </c>
+      <c r="J41" t="inlineStr"/>
+      <c r="K41" t="inlineStr"/>
+      <c r="L41" t="inlineStr"/>
+      <c r="M41" t="inlineStr"/>
+      <c r="N41" t="inlineStr"/>
       <c r="O41" t="inlineStr">
         <is>
           <t>ok</t>
@@ -3021,11 +3001,7 @@
           <t>good</t>
         </is>
       </c>
-      <c r="Q41" t="inlineStr">
-        <is>
-          <t>fail</t>
-        </is>
-      </c>
+      <c r="Q41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -3035,7 +3011,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>features: Cherry MX Speed, 4000 Hz polling, aluminum frame; capacity: large</t>
+          <t>features: Cherry MX Speed, 4000 Hz polling, aluminum frame; capacity: large</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -3050,46 +3026,26 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Elevate your gaming experience with the Corsair K100 RGB Keyboard. Boasting a robust aluminum frame and Cherry MX Speed switches for lightning-fast actuation, this keyboard is designed for high-performance gaming. With 4000 Hz polling for seamless key registration, you'll enjoy precise control and a competitive edge. The large capacity ensures a spacious typing experience, while the brushed aluminum finish adds a touch of premium style. Backed by a 2-year warranty, this keyboard is built to last.</t>
+          <t>Elevate your gaming experience with the Corsair K100 RGB Keyboard, engineered for speed and precision. Its aluminum frame provides a sturdy base, while the Cherry MX Speed switches deliver rapid actuation and tactile feedback. With 4000 Hz polling, you'll enjoy seamless key registration and responsive performance. Durable and built to last, this keyboard is backed by a 2-year warranty. Perfect for gamers seeking a high-performance typing experience.</t>
         </is>
       </c>
       <c r="F42" t="n">
-        <v>4072</v>
+        <v>2587.3</v>
       </c>
       <c r="G42" t="n">
         <v>205</v>
       </c>
       <c r="H42" t="n">
-        <v>100</v>
+        <v>89</v>
       </c>
       <c r="I42" t="n">
-        <v>1.01e-05</v>
-      </c>
-      <c r="J42" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="K42" t="inlineStr">
-        <is>
-          <t>good</t>
-        </is>
-      </c>
-      <c r="L42" t="inlineStr">
-        <is>
-          <t>good</t>
-        </is>
-      </c>
-      <c r="M42" t="inlineStr">
-        <is>
-          <t>good</t>
-        </is>
-      </c>
-      <c r="N42" t="inlineStr">
-        <is>
-          <t>bad</t>
-        </is>
-      </c>
+        <v>9.439999999999999e-06</v>
+      </c>
+      <c r="J42" t="inlineStr"/>
+      <c r="K42" t="inlineStr"/>
+      <c r="L42" t="inlineStr"/>
+      <c r="M42" t="inlineStr"/>
+      <c r="N42" t="inlineStr"/>
       <c r="O42" t="inlineStr">
         <is>
           <t>ok</t>
@@ -3100,16 +3056,12 @@
           <t>good</t>
         </is>
       </c>
-      <c r="Q42" t="inlineStr">
-        <is>
-          <t>fail</t>
-        </is>
-      </c>
+      <c r="Q42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Logitech MX Master 3S</t>
+          <t>Logitech MX Master 3S</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -3129,46 +3081,26 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Elevate your productivity with the Logitech MX Master 3S. This advanced mouse boasts an 8K DPI sensor for precise navigation and a MagSpeed scroll wheel for effortless zooming. Enjoy seamless connectivity with both Bolt and Bluetooth options. Available in multiple colors to match your style, this mouse is crafted from durable plastic. Backed by a 1-year limited warranty, you can trust the Logitech MX Master 3S to deliver reliable performance and comfort.</t>
+          <t>Experience precision and speed with the Logitech MX Master 3S. This advanced mouse boasts an 8K DPI sensor, ensuring accurate tracking and effortless navigation. The MagSpeed scroll wheel lets you zoom and scroll with ease, while Bolt and Bluetooth connectivity options provide reliable and lag-free performance. Available in multiple color options, this mouse is designed to fit your style. With a 1-year limited warranty, you can trust your investment in precision and performance.</t>
         </is>
       </c>
       <c r="F43" t="n">
-        <v>3306.6</v>
+        <v>2799.3</v>
       </c>
       <c r="G43" t="n">
         <v>207</v>
       </c>
       <c r="H43" t="n">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="I43" t="n">
-        <v>9.840000000000001e-06</v>
-      </c>
-      <c r="J43" t="inlineStr">
-        <is>
-          <t>good</t>
-        </is>
-      </c>
-      <c r="K43" t="inlineStr">
-        <is>
-          <t>good</t>
-        </is>
-      </c>
-      <c r="L43" t="inlineStr">
-        <is>
-          <t>good</t>
-        </is>
-      </c>
-      <c r="M43" t="inlineStr">
-        <is>
-          <t>good</t>
-        </is>
-      </c>
-      <c r="N43" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
+        <v>9.660000000000001e-06</v>
+      </c>
+      <c r="J43" t="inlineStr"/>
+      <c r="K43" t="inlineStr"/>
+      <c r="L43" t="inlineStr"/>
+      <c r="M43" t="inlineStr"/>
+      <c r="N43" t="inlineStr"/>
       <c r="O43" t="inlineStr">
         <is>
           <t>ok</t>
@@ -3179,11 +3111,7 @@
           <t>good</t>
         </is>
       </c>
-      <c r="Q43" t="inlineStr">
-        <is>
-          <t>pass</t>
-        </is>
-      </c>
+      <c r="Q43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -3193,7 +3121,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>features: 63 g ultralight, 30K DPI Focus Pro sensor; battery: long‑lasting</t>
+          <t>features: 63 g ultralight, 30K DPI Focus Pro sensor; battery: long‑lasting</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -3208,46 +3136,26 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Take your gaming to the next level with the Razer DeathAdder V3 Pro. Weighing in at just 63 grams, this ultralight mouse is designed for marathon gaming sessions. The 30K DPI Focus Pro sensor provides unparalleled accuracy and speed. Plus, its long-lasting battery ensures you can play without interruption. Crafted from durable plastic, the DeathAdder V3 Pro is built to last. Backed by a 2-year warranty, you can trust it to deliver top-notch performance. Upgrade your gaming experience today.</t>
+          <t>Take your gaming to the next level with the Razer DeathAdder V3 Pro. Weighing in at just 63 grams, this ultralight mouse glides effortlessly across any surface. The 30K DPI Focus Pro sensor provides pinpoint accuracy, while the long-lasting battery keeps you gaming for hours on end. Built with durable plastic, this mouse is designed to withstand the rigors of intense gaming sessions. Backed by a 2-year warranty, you can trust that your DeathAdder V3 Pro will deliver top-notch performance for years to come.</t>
         </is>
       </c>
       <c r="F44" t="n">
-        <v>4700.8</v>
+        <v>2806.2</v>
       </c>
       <c r="G44" t="n">
         <v>210</v>
       </c>
       <c r="H44" t="n">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="I44" t="n">
-        <v>1.09e-05</v>
-      </c>
-      <c r="J44" t="inlineStr">
-        <is>
-          <t>good</t>
-        </is>
-      </c>
-      <c r="K44" t="inlineStr">
-        <is>
-          <t>good</t>
-        </is>
-      </c>
-      <c r="L44" t="inlineStr">
-        <is>
-          <t>good</t>
-        </is>
-      </c>
-      <c r="M44" t="inlineStr">
-        <is>
-          <t>good</t>
-        </is>
-      </c>
-      <c r="N44" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
+        <v>1.11e-05</v>
+      </c>
+      <c r="J44" t="inlineStr"/>
+      <c r="K44" t="inlineStr"/>
+      <c r="L44" t="inlineStr"/>
+      <c r="M44" t="inlineStr"/>
+      <c r="N44" t="inlineStr"/>
       <c r="O44" t="inlineStr">
         <is>
           <t>ok</t>
@@ -3258,21 +3166,17 @@
           <t>good</t>
         </is>
       </c>
-      <c r="Q44" t="inlineStr">
-        <is>
-          <t>pass</t>
-        </is>
-      </c>
+      <c r="Q44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Samsung 980 Pro 2 TB NVMe SSD</t>
+          <t>Samsung 980 Pro 2 TB NVMe SSD</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>features: PCIe 4.0, up to 7 000 MB/s read, nickel coating; battery: long‑lasting</t>
+          <t>features: PCIe 4.0, up to 7 000 MB/s read, nickel coating; battery: long‑lasting</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -3287,20 +3191,20 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Take your gaming and content creation to the next level with the Samsung 980 Pro 2TB NVMe SSD. Boasting incredible speeds of up to 7,000 MB/s read, this PCIe 4.0 drive ensures seamless performance and rapid loading times. With a long-lasting battery and durable nickel coating, you can rely on it for years to come. Built with high-quality PCB and NAND flash materials, this SSD is designed to deliver exceptional reliability and speed. Backed by a 5-year limited warranty, you can trust that your investment is protected.</t>
+          <t>Take your gaming and content creation to the next level with the Samsung 980 Pro 2 TB NVMe SSD. Boasting incredible speeds of up to 7,000 MB/s read, this PCIe 4.0 drive ensures seamless performance and rapid loading times. With its long-lasting battery and durable nickel coating, you can trust it to keep up with your demanding needs. Backed by a 5-year limited warranty, this SSD is built to last and deliver exceptional results.</t>
         </is>
       </c>
       <c r="F45" t="n">
-        <v>3723.5</v>
+        <v>2595.6</v>
       </c>
       <c r="G45" t="n">
         <v>221</v>
       </c>
       <c r="H45" t="n">
-        <v>114</v>
+        <v>97</v>
       </c>
       <c r="I45" t="n">
-        <v>1.13e-05</v>
+        <v>1.024e-05</v>
       </c>
       <c r="J45" t="inlineStr"/>
       <c r="K45" t="inlineStr"/>
@@ -3322,7 +3226,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Seagate Portable 5 TB HDD</t>
+          <t>Seagate Portable 5 TB HDD</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -3342,20 +3246,20 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Store and transport your files with ease using the Seagate Portable 5 TB HDD. This compact drive features a 2.5" form factor and plug-and-play functionality via USB 3.0, making it simple to get started. With a 4.7-star rating from satisfied customers, you can trust this reliable storage solution. The durable plastic shell protects your data, and a 1-year limited warranty provides peace of mind.</t>
+          <t>Store and transport your massive digital library with ease using the Seagate Portable 5 TB HDD. This compact drive features a plug-and-play USB 3.0 connection, making it simple to get started. With a 2.5" form factor, it's the perfect size for on-the-go use. Backed by a 4.7-star rating and a 1-year limited warranty, you can trust this reliable external hard drive to safeguard your files.</t>
         </is>
       </c>
       <c r="F46" t="n">
-        <v>4707.4</v>
+        <v>2741.6</v>
       </c>
       <c r="G46" t="n">
         <v>219</v>
       </c>
       <c r="H46" t="n">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="I46" t="n">
-        <v>9.72e-06</v>
+        <v>1.002e-05</v>
       </c>
       <c r="J46" t="inlineStr"/>
       <c r="K46" t="inlineStr"/>
@@ -3377,12 +3281,12 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>SanDisk Extreme PRO 128 GB SDXC</t>
+          <t>SanDisk Extreme PRO 128 GB SDXC</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>features: UHS‑I U3, 200 MB/s read, waterproof; battery: long‑lasting</t>
+          <t>features: UHS‑I U3, 200 MB/s read, waterproof; battery: long‑lasting</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -3397,20 +3301,20 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Capture life's most epic moments with the SanDisk Extreme PRO 128 GB SDXC card. With blazing-fast UHS-I U3 speeds of up to 200 MB/s read, you'll never miss a shot. Plus, its waterproof design ensures your memories stay safe, even in the most rugged conditions. And with a long-lasting battery, you can keep shooting without interruption. Backed by a lifetime limited warranty, this card is the ultimate companion for your adventures.</t>
+          <t>Capture life's most epic moments with the SanDisk Extreme PRO 128 GB SDXC card. With UHS-I U3 speeds of up to 200 MB/s read, you can quickly transfer and store stunning 4K and Full HD footage. Rugged and reliable, this card withstands water, dust, and extreme temperatures, ensuring your memories stay safe. Plus, its long-lasting battery means you can shoot all day without interruption. Backed by a lifetime limited warranty, you can trust your memories are protected.</t>
         </is>
       </c>
       <c r="F47" t="n">
-        <v>3428.6</v>
+        <v>3359.6</v>
       </c>
       <c r="G47" t="n">
         <v>210</v>
       </c>
       <c r="H47" t="n">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="I47" t="n">
-        <v>9.9e-06</v>
+        <v>1.05e-05</v>
       </c>
       <c r="J47" t="inlineStr"/>
       <c r="K47" t="inlineStr"/>
@@ -3432,12 +3336,12 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Kingston Fury Beast 32 GB DDR5</t>
+          <t>Kingston Fury Beast 32 GB DDR5</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>features: 6000 MT/s, Intel XMP 3.0, low‑profile heat spreader; energy efficient</t>
+          <t>features: 6000 MT/s, Intel XMP 3.0, low‑profile heat spreader; energy efficient</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -3452,20 +3356,20 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Boost your system's performance with the Kingston Fury Beast 32 GB DDR5 memory kit. With speeds of up to 6000 MT/s, you'll experience lightning-fast data transfer and improved multitasking capabilities. The low-profile heat spreader ensures efficient cooling, while Intel XMP 3.0 support makes it easy to optimize your system. Plus, the aluminum heatspreader provides durability. Backed by a lifetime warranty, this kit is a reliable choice for gamers and content creators alike.</t>
+          <t>Upgrade your gaming experience with the Kingston Fury Beast 32 GB DDR5 RAM. This high-performance memory module boasts speeds of 6000 MT/s, ensuring seamless multitasking and fast loading times. With Intel XMP 3.0, you can easily optimize settings for maximum performance. The low-profile heat spreader keeps your system cool, while the aluminum material provides durability. Backed by a lifetime warranty, the Fury Beast 32 GB DDR5 is a reliable choice for gamers and content creators alike.</t>
         </is>
       </c>
       <c r="F48" t="n">
-        <v>3605.5</v>
+        <v>2053.1</v>
       </c>
       <c r="G48" t="n">
         <v>214</v>
       </c>
       <c r="H48" t="n">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="I48" t="n">
-        <v>1.03e-05</v>
+        <v>1.04e-05</v>
       </c>
       <c r="J48" t="inlineStr"/>
       <c r="K48" t="inlineStr"/>
@@ -3492,7 +3396,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>features: 2560×1440 170 Hz IPS, HDR400, G‑Sync Compatible; capacity: large</t>
+          <t>features: 2560×1440 170 Hz IPS, HDR400, G‑Sync Compatible; capacity: large</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -3507,20 +3411,20 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Elevate your gaming experience with the Acer Predator XB273U 27" Monitor. Boasting a stunning 2560x1440 resolution and 170Hz refresh rate, this IPS panel delivers crisp visuals and seamless motion. HDR400 and G-Sync Compatible ensure immersive color and reduced screen tearing. Built to last with a sturdy plastic and metal stand, this monitor is designed to withstand intense gaming sessions. Backed by a 3-year warranty, you can focus on your game, not your gear.</t>
+          <t>Elevate your gaming experience with the Acer Predator XB273U 27" Monitor. Boasting a crystal-clear 2560x1440 resolution and 170Hz refresh rate, this IPS display delivers seamless visuals. HDR400 technology enhances color accuracy, while G-Sync Compatible ensures a silky-smooth gaming experience. With its sturdy plastic and metal stand, this large monitor is built to last. Backed by a 3-year warranty, you can focus on your game, not maintenance.</t>
         </is>
       </c>
       <c r="F49" t="n">
-        <v>3600.4</v>
+        <v>2247.3</v>
       </c>
       <c r="G49" t="n">
         <v>216</v>
       </c>
       <c r="H49" t="n">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="I49" t="n">
-        <v>1.05e-05</v>
+        <v>1.032e-05</v>
       </c>
       <c r="J49" t="inlineStr"/>
       <c r="K49" t="inlineStr"/>
@@ -3547,7 +3451,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>features: 4K UHD IPS, 98% P3, Thunderbolt 3; color options: multiple</t>
+          <t>features: 4K UHD IPS, 98% P3, Thunderbolt 3; color options: multiple</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -3562,20 +3466,20 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Experience breathtaking visuals on the BenQ PD2725U 27" Monitor, boasting a stunning 4K UHD IPS display that covers 98% of the P3 color space. With Thunderbolt 3 connectivity, you can transfer data at incredible speeds. The durable metal stand ensures a sturdy base, while the multiple color options allow you to personalize your workspace. Backed by a comprehensive 3-year warranty, this monitor is designed to deliver exceptional performance and reliability for years to come.</t>
+          <t>Elevate your visual experience with the BenQ PD2725U 27" Monitor. This stunning 4K UHD IPS display boasts 98% P3 color accuracy, ensuring vibrant and lifelike colors. With Thunderbolt 3 connectivity, you can easily transfer data and power your devices. The durable metal stand provides a sturdy base, while the multiple color options allow you to customize the look to fit your workspace. Backed by a 3-year warranty, this monitor is a reliable choice for professionals and creatives alike.</t>
         </is>
       </c>
       <c r="F50" t="n">
-        <v>4163</v>
+        <v>2770.3</v>
       </c>
       <c r="G50" t="n">
         <v>214</v>
       </c>
       <c r="H50" t="n">
-        <v>100</v>
+        <v>110</v>
       </c>
       <c r="I50" t="n">
-        <v>1.03e-05</v>
+        <v>1.088e-05</v>
       </c>
       <c r="J50" t="inlineStr"/>
       <c r="K50" t="inlineStr"/>
@@ -3617,20 +3521,20 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Elevate your creative workflow with the ASUS ProArt PA278QV Monitor. This 27" IPS display boasts vibrant colors, with 100% sRGB coverage and Calman Verified accuracy. Perfect for graphic designers, photographers, and videographers, it ensures precise color representation. The sturdy metal stand keeps the monitor stable, while its light weight makes it easy to reposition. With a 3-year warranty, you can focus on your craft, knowing your investment is protected.</t>
+          <t>Elevate your creative workflow with the ASUS ProArt PA278QV Monitor. This 27" IPS display boasts stunning 2560x1440 resolution and 100% sRGB color accuracy, ensuring vibrant and true-to-life visuals. Calman Verified for precision, this monitor is perfect for graphic designers, photographers, and videographers. Plus, its light weight and sturdy metal stand make it easy to position and adjust. Backed by a 3-year warranty, you can trust your creative endeavors are in good hands.</t>
         </is>
       </c>
       <c r="F51" t="n">
-        <v>4679.7</v>
+        <v>4027.6</v>
       </c>
       <c r="G51" t="n">
         <v>214</v>
       </c>
       <c r="H51" t="n">
-        <v>98</v>
+        <v>107</v>
       </c>
       <c r="I51" t="n">
-        <v>1.02e-05</v>
+        <v>1.07e-05</v>
       </c>
       <c r="J51" t="inlineStr"/>
       <c r="K51" t="inlineStr"/>

</xml_diff>